<commit_message>
feat(reports): save reports into dated subfolders and support discovery in UI\n\n- add get_dated_reports_dir helper\n- write price_tracker, compare_scans, dashboard_generator to dated folders\n- update web panel to scan dated folders\n(keeps backwards-compatible read behavior)
</commit_message>
<xml_diff>
--- a/data/mappings/pricing_sample.xlsx
+++ b/data/mappings/pricing_sample.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jalil Shojazade\Desktop\Luxbaz_product_import\02_Product_processor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Luxbaz\All Codes\Projects\product-import-pipeline\data\mappings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1F19E2-E9E7-4D6B-AFFD-32918E06A31D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A79B9EC-E738-4B2C-861A-99C170681B39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -442,7 +442,7 @@
         <v>15</v>
       </c>
       <c r="D3" s="2">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>